<commit_message>
Regenerate birds xlsx from the renamed JSON
The previous commit's -x doc build did not rewrite ro-crate-metadata.xlsx,
so the spreadsheet still described the classes under their old names. That
matters beyond tidiness: generate-masp-docs -x syncs from whichever of the
JSON/xlsx pair is newer, so a later build with a freshly touched xlsx would
have reverted the renames.

Runs rocxl --JSON over the profile crate to rebuild the spreadsheet (and its
ro-crate-preview.html) from the JSON. rocxl also reorders entities and bumps
dateModified in the JSON — no entities added or dropped, 61 either side.

Re-verified after the round trip: example crate validates with 0 errors and
6 class rules matched, and the root class still resolves to
RepositoryCollection through getRootDatasetTypes()/getEnabledClasses().

Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/birds/profile-crate/ro-crate-metadata.xlsx
+++ b/birds/profile-crate/ro-crate-metadata.xlsx
@@ -23,7 +23,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="433" uniqueCount="244">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="448" uniqueCount="255">
   <si>
     <t>Name</t>
   </si>
@@ -34,7 +34,7 @@
     <t>@id</t>
   </si>
   <si>
-    <t>https://language-research-technology.github.io/ro-crate-masp/profiles/birds/profile-crate/</t>
+    <t>https://benfoley.github.io/masp-profiles/birds/profile-crate/</t>
   </si>
   <si>
     <t>@type</t>
@@ -88,13 +88,13 @@
     <t>hasResource</t>
   </si>
   <si>
-    <t>["#hasSpecializedSchema", "#hasExampleCrate", "#hasGuidance", "#hasConformanceIndicators"]</t>
+    <t>["#hasSpecializedSchema", "#hasExampleCrate", "#hasGuidance", "#hasEditorMode", "#hasConformanceIndicators"]</t>
   </si>
   <si>
     <t>hasPart</t>
   </si>
   <si>
-    <t>["profile-documentation.md", "examples/birds-crate/ro-crate-metadata.json"]</t>
+    <t>["profile-documentation.md", "crate-o-mode.json", "examples/birds-crate/ro-crate-metadata.json"]</t>
   </si>
   <si>
     <t>ldac</t>
@@ -121,7 +121,7 @@
     <t/>
   </si>
   <si>
-    <t>["index.html", "profile-documentation.md", "examples"]</t>
+    <t>["index.html", "profile-documentation.md", "examples", "crate-o-mode.json"]</t>
   </si>
   <si>
     <t>encodingFormat</t>
@@ -145,10 +145,25 @@
     <t>["https://www.nationalarchives.gov.uk/PRONOM/fmt/1149", text/markdown]</t>
   </si>
   <si>
-    <t>"https://language-research-technology.github.io/ro-crate-masp/profiles/birds/profile-crate/"</t>
-  </si>
-  <si>
-    <t>2026-08-07T17:45:15+10:00</t>
+    <t>"https://benfoley.github.io/masp-profiles/birds/profile-crate/"</t>
+  </si>
+  <si>
+    <t>2026-08-07T18:27:45+10:00</t>
+  </si>
+  <si>
+    <t>crate-o-mode.json</t>
+  </si>
+  <si>
+    <t>Resource2Crate config file</t>
+  </si>
+  <si>
+    <t>Mini Crate-O mode file for this profile (root dataset types, input groups and long-text inputs — the schema/grammar is provided by the MASP profile crate itself). No `buildOptions` yet.</t>
+  </si>
+  <si>
+    <t>["https://www.nationalarchives.gov.uk/PRONOM/fmt/817", application/json]</t>
+  </si>
+  <si>
+    <t>2026-08-07T18:00:42+10:00</t>
   </si>
   <si>
     <t>examples/birds-crate/ro-crate-metadata.json</t>
@@ -202,7 +217,7 @@
     <t>https://language-research-technology.github.io/ro-crate-masp/profiles/ro-crate-masp/profile-crate/</t>
   </si>
   <si>
-    <t>https://language-research-technology.github.io/ro-crate-masp/profiles/birds/profile-crate/#profile</t>
+    <t>https://benfoley.github.io/masp-profiles/birds/profile-crate/#profile</t>
   </si>
   <si>
     <t>hasRole</t>
@@ -250,6 +265,18 @@
     <t>"profile-documentation.md"</t>
   </si>
   <si>
+    <t>#hasEditorMode</t>
+  </si>
+  <si>
+    <t>Editor Mode / Build Workflow</t>
+  </si>
+  <si>
+    <t>"https://w3id.org/ro/mode"</t>
+  </si>
+  <si>
+    <t>"crate-o-mode.json"</t>
+  </si>
+  <si>
     <t>#hasConformanceIndicators</t>
   </si>
   <si>
@@ -289,61 +316,58 @@
     <t>#Class_Collection</t>
   </si>
   <si>
-    <t>Collection</t>
+    <t>RepositoryCollection</t>
   </si>
   <si>
     <t>["http://schema.org/Dataset", "http://pcdm.org/models#Collection"]</t>
   </si>
   <si>
-    <t>The Root Data Entity. A Collection groups the bird entries (Objects) that make up the site. It MUST be typed `["Dataset", "RepositoryCollection"]`.</t>
+    <t>The Collection — the Root Data Entity. It groups the bird entries (Objects) that make up the site, and MUST be typed `["Dataset", "RepositoryCollection"]`.</t>
   </si>
   <si>
     <t>#Class_Object</t>
   </si>
   <si>
-    <t>Object</t>
+    <t>RepositoryObject</t>
   </si>
   <si>
     <t>"http://pcdm.org/models#Object"</t>
   </si>
   <si>
-    <t>A member of the Collection: one bird entry, gathering the name, story, speaker and media files for a single bird. Typed `RepositoryObject`.</t>
+    <t>An Object — a member of the Collection: one bird entry, gathering the name, story, speaker and media files for a single bird.</t>
   </si>
   <si>
     <t>#Class_Speaker</t>
   </si>
   <si>
-    <t>Speaker</t>
+    <t>Person</t>
   </si>
   <si>
     <t>"http://schema.org/Person"</t>
   </si>
   <si>
-    <t>The person heard in an Object's recordings. `ldac:speaker` also permits an `Organization`; this profile requires a `Person`.</t>
+    <t>The Speaker — the person heard in an Object's recordings, linked with `ldac:speaker`. That term also permits an `Organization`; this profile requires a `Person`.</t>
   </si>
   <si>
     <t>#Class_File</t>
   </si>
   <si>
-    <t>Media File</t>
-  </si>
-  <si>
     <t>"http://schema.org/MediaObject"</t>
   </si>
   <si>
-    <t>An image or audio file in the crate. Media files that belong to a bird entry link back to it with `isPartOf`.</t>
+    <t>A Media File — an image or audio file in the crate. Media files that belong to a bird entry link back to it with `isPartOf`.</t>
   </si>
   <si>
     <t>#Class_AboutPage</t>
   </si>
   <si>
-    <t>About Page</t>
+    <t>AboutPage</t>
   </si>
   <si>
     <t>["http://schema.org/MediaObject", "http://schema.org/AboutPage"]</t>
   </si>
   <si>
-    <t>An optional Markdown file typed `["File", "AboutPage"]` holding prose about the Collection. The static site generator renders it as the site's About page.</t>
+    <t>The About Page — an optional Markdown file typed `["File", "AboutPage"]` holding prose about the Collection. The static site generator renders it as the site's About page.</t>
   </si>
   <si>
     <t>rdfs:label</t>
@@ -673,7 +697,7 @@
     <t>The Collection must declare conformance to this profile or to the LDAC Collection profile.</t>
   </si>
   <si>
-    <t>["https://language-research-technology.github.io/ro-crate-masp/profiles/birds/profile-crate/#profile", "https://w3id.org/ldac/profile#Collection"]</t>
+    <t>["https://benfoley.github.io/masp-profiles/birds/profile-crate/#profile", "https://w3id.org/ldac/profile#Collection"]</t>
   </si>
   <si>
     <t>#propertyValue_licenseUrl</t>
@@ -724,31 +748,40 @@
     <t>Canonical identifiers that indicate conformance to this profile.</t>
   </si>
   <si>
-    <t>"https://language-research-technology.github.io/ro-crate-masp/profiles/birds/profile-crate/#profile"</t>
+    <t>"https://benfoley.github.io/masp-profiles/birds/profile-crate/#profile"</t>
+  </si>
+  <si>
+    <t>https://w3id.org/ro/mode</t>
+  </si>
+  <si>
+    <t>DefinedTerm</t>
+  </si>
+  <si>
+    <t>Editor Mode</t>
+  </si>
+  <si>
+    <t>Role indicating a resource is an editor configuration mode file.</t>
   </si>
   <si>
     <t>https://w3id.org/ro/conformance-indicators</t>
   </si>
   <si>
-    <t>DefinedTerm</t>
-  </si>
-  <si>
     <t>Role indicating a resource enumerates identifiers that are accepted as conformance indicators for the profile.</t>
   </si>
   <si>
+    <t>https://www.nationalarchives.gov.uk/PRONOM/fmt/817</t>
+  </si>
+  <si>
+    <t>DigitalFormat</t>
+  </si>
+  <si>
+    <t>JSON Data Interchange Format</t>
+  </si>
+  <si>
     <t>https://www.nationalarchives.gov.uk/PRONOM/fmt/1149</t>
   </si>
   <si>
-    <t>DigitalFormat</t>
-  </si>
-  <si>
     <t>Markdown</t>
-  </si>
-  <si>
-    <t>https://www.nationalarchives.gov.uk/PRONOM/fmt/817</t>
-  </si>
-  <si>
-    <t>JSON Data Interchange Format</t>
   </si>
   <si>
     <t>https://www.nationalarchives.gov.uk/PRONOM/fmt/471</t>
@@ -1262,30 +1295,30 @@
         <v>8</v>
       </c>
       <c r="E1" t="s">
-        <v>203</v>
+        <v>211</v>
       </c>
       <c r="F1" t="s">
-        <v>80</v>
+        <v>89</v>
       </c>
       <c r="G1" t="s">
-        <v>81</v>
+        <v>90</v>
       </c>
     </row>
     <row r="2" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
-        <v>204</v>
+        <v>212</v>
       </c>
       <c r="B2" t="s">
-        <v>205</v>
+        <v>213</v>
       </c>
       <c r="C2" t="s">
-        <v>206</v>
+        <v>214</v>
       </c>
       <c r="D2" t="s">
-        <v>207</v>
+        <v>215</v>
       </c>
       <c r="E2" t="s">
-        <v>208</v>
+        <v>216</v>
       </c>
       <c r="F2">
         <v>1</v>
@@ -1296,19 +1329,19 @@
     </row>
     <row r="3" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
-        <v>209</v>
+        <v>217</v>
       </c>
       <c r="B3" t="s">
-        <v>205</v>
+        <v>213</v>
       </c>
       <c r="C3" t="s">
-        <v>210</v>
+        <v>218</v>
       </c>
       <c r="D3" t="s">
-        <v>211</v>
+        <v>219</v>
       </c>
       <c r="E3" t="s">
-        <v>212</v>
+        <v>220</v>
       </c>
       <c r="F3">
         <v>1</v>
@@ -1319,19 +1352,19 @@
     </row>
     <row r="4" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
+        <v>221</v>
+      </c>
+      <c r="B4" t="s">
         <v>213</v>
       </c>
-      <c r="B4" t="s">
-        <v>205</v>
-      </c>
       <c r="C4" t="s">
-        <v>214</v>
+        <v>222</v>
       </c>
       <c r="D4" t="s">
-        <v>215</v>
+        <v>223</v>
       </c>
       <c r="E4" t="s">
-        <v>216</v>
+        <v>224</v>
       </c>
       <c r="F4">
         <v>1</v>
@@ -1339,19 +1372,19 @@
     </row>
     <row r="5" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
-        <v>217</v>
+        <v>225</v>
       </c>
       <c r="B5" t="s">
-        <v>205</v>
+        <v>213</v>
       </c>
       <c r="C5" t="s">
-        <v>218</v>
+        <v>226</v>
       </c>
       <c r="D5" t="s">
-        <v>219</v>
+        <v>227</v>
       </c>
       <c r="E5" t="s">
-        <v>220</v>
+        <v>228</v>
       </c>
       <c r="F5">
         <v>1</v>
@@ -1362,19 +1395,19 @@
     </row>
     <row r="6" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
-        <v>221</v>
+        <v>229</v>
       </c>
       <c r="B6" t="s">
-        <v>205</v>
+        <v>213</v>
       </c>
       <c r="C6" t="s">
-        <v>222</v>
+        <v>230</v>
       </c>
       <c r="D6" t="s">
-        <v>223</v>
+        <v>231</v>
       </c>
       <c r="E6" t="s">
-        <v>224</v>
+        <v>232</v>
       </c>
       <c r="F6">
         <v>1</v>
@@ -1411,41 +1444,41 @@
         <v>8</v>
       </c>
       <c r="E1" t="s">
-        <v>225</v>
+        <v>233</v>
       </c>
     </row>
     <row r="2" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
-        <v>226</v>
+        <v>234</v>
       </c>
       <c r="B2" t="s">
-        <v>227</v>
+        <v>235</v>
       </c>
       <c r="C2" t="s">
-        <v>228</v>
+        <v>236</v>
       </c>
       <c r="D2" t="s">
-        <v>229</v>
+        <v>237</v>
       </c>
       <c r="E2" t="s">
-        <v>216</v>
+        <v>224</v>
       </c>
     </row>
     <row r="3" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
-        <v>230</v>
+        <v>238</v>
       </c>
       <c r="B3" t="s">
-        <v>227</v>
+        <v>235</v>
       </c>
       <c r="C3" t="s">
-        <v>231</v>
+        <v>239</v>
       </c>
       <c r="D3" t="s">
-        <v>232</v>
+        <v>240</v>
       </c>
       <c r="E3" t="s">
-        <v>233</v>
+        <v>241</v>
       </c>
     </row>
   </sheetData>
@@ -1456,7 +1489,7 @@
 
 <file path=xl/worksheets/sheet12.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:D2"/>
+  <dimension ref="A1:D3"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <cols>
     <col min="1" max="4" width="20" customWidth="1"/>
@@ -1478,16 +1511,30 @@
     </row>
     <row r="2" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
-        <v>234</v>
+        <v>242</v>
       </c>
       <c r="B2" t="s">
-        <v>235</v>
+        <v>243</v>
       </c>
       <c r="C2" t="s">
-        <v>76</v>
+        <v>244</v>
       </c>
       <c r="D2" t="s">
-        <v>236</v>
+        <v>245</v>
+      </c>
+    </row>
+    <row r="3" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A3" t="s">
+        <v>246</v>
+      </c>
+      <c r="B3" t="s">
+        <v>243</v>
+      </c>
+      <c r="C3" t="s">
+        <v>85</v>
+      </c>
+      <c r="D3" t="s">
+        <v>247</v>
       </c>
     </row>
   </sheetData>
@@ -1517,35 +1564,35 @@
     </row>
     <row r="2" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
-        <v>237</v>
+        <v>248</v>
       </c>
       <c r="B2" t="s">
-        <v>238</v>
+        <v>249</v>
       </c>
       <c r="C2" t="s">
-        <v>239</v>
+        <v>250</v>
       </c>
     </row>
     <row r="3" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
-        <v>240</v>
+        <v>251</v>
       </c>
       <c r="B3" t="s">
-        <v>238</v>
+        <v>249</v>
       </c>
       <c r="C3" t="s">
-        <v>241</v>
+        <v>252</v>
       </c>
     </row>
     <row r="4" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
-        <v>242</v>
+        <v>253</v>
       </c>
       <c r="B4" t="s">
-        <v>238</v>
+        <v>249</v>
       </c>
       <c r="C4" t="s">
-        <v>243</v>
+        <v>254</v>
       </c>
     </row>
   </sheetData>
@@ -1643,7 +1690,7 @@
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:G4"/>
+  <dimension ref="A1:G5"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <cols>
     <col min="1" max="7" width="20" customWidth="1"/>
@@ -1695,7 +1742,7 @@
         <v>41</v>
       </c>
     </row>
-    <row r="3" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
         <v>42</v>
       </c>
@@ -1711,24 +1758,44 @@
       <c r="E3" t="s">
         <v>45</v>
       </c>
-    </row>
-    <row r="4" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="G3" t="s">
+        <v>46</v>
+      </c>
+    </row>
+    <row r="4" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
-        <v>46</v>
+        <v>47</v>
       </c>
       <c r="B4" t="s">
         <v>37</v>
       </c>
       <c r="C4" t="s">
-        <v>46</v>
+        <v>48</v>
       </c>
       <c r="D4" t="s">
+        <v>49</v>
+      </c>
+      <c r="E4" t="s">
+        <v>50</v>
+      </c>
+    </row>
+    <row r="5" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A5" t="s">
+        <v>51</v>
+      </c>
+      <c r="B5" t="s">
+        <v>37</v>
+      </c>
+      <c r="C5" t="s">
+        <v>51</v>
+      </c>
+      <c r="D5" t="s">
         <v>31</v>
       </c>
-      <c r="E4" t="s">
-        <v>47</v>
-      </c>
-      <c r="G4" t="s">
+      <c r="E5" t="s">
+        <v>52</v>
+      </c>
+      <c r="G5" t="s">
         <v>41</v>
       </c>
     </row>
@@ -1759,13 +1826,13 @@
     </row>
     <row r="2" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
-        <v>48</v>
+        <v>53</v>
       </c>
       <c r="B2" t="s">
-        <v>49</v>
+        <v>54</v>
       </c>
       <c r="C2" t="s">
-        <v>50</v>
+        <v>55</v>
       </c>
     </row>
   </sheetData>
@@ -1796,43 +1863,43 @@
         <v>8</v>
       </c>
       <c r="E1" t="s">
-        <v>51</v>
+        <v>56</v>
       </c>
     </row>
     <row r="2" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
-        <v>52</v>
+        <v>57</v>
       </c>
       <c r="B2" t="s">
-        <v>53</v>
+        <v>58</v>
       </c>
       <c r="C2" t="s">
-        <v>54</v>
+        <v>59</v>
       </c>
       <c r="D2" t="s">
-        <v>55</v>
+        <v>60</v>
       </c>
     </row>
     <row r="3" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
-        <v>56</v>
+        <v>61</v>
       </c>
       <c r="B3" t="s">
-        <v>53</v>
+        <v>58</v>
       </c>
       <c r="C3" t="s">
-        <v>57</v>
+        <v>62</v>
       </c>
       <c r="E3" t="s">
-        <v>58</v>
+        <v>63</v>
       </c>
     </row>
     <row r="4" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
-        <v>59</v>
+        <v>64</v>
       </c>
       <c r="B4" t="s">
-        <v>53</v>
+        <v>58</v>
       </c>
       <c r="C4" t="s">
         <v>7</v>
@@ -1849,7 +1916,7 @@
 
 <file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:F5"/>
+  <dimension ref="A1:F6"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <cols>
     <col min="1" max="6" width="20" customWidth="1"/>
@@ -1866,81 +1933,98 @@
         <v>6</v>
       </c>
       <c r="D1" t="s">
-        <v>60</v>
+        <v>65</v>
       </c>
       <c r="E1" t="s">
         <v>22</v>
       </c>
       <c r="F1" t="s">
-        <v>61</v>
+        <v>66</v>
       </c>
     </row>
     <row r="2" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
-        <v>62</v>
+        <v>67</v>
       </c>
       <c r="B2" t="s">
-        <v>63</v>
+        <v>68</v>
       </c>
       <c r="C2" t="s">
-        <v>64</v>
+        <v>69</v>
       </c>
       <c r="D2" t="s">
-        <v>65</v>
+        <v>70</v>
       </c>
       <c r="E2" t="s">
-        <v>66</v>
+        <v>71</v>
       </c>
     </row>
     <row r="3" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
-        <v>67</v>
+        <v>72</v>
       </c>
       <c r="B3" t="s">
-        <v>63</v>
+        <v>68</v>
       </c>
       <c r="C3" t="s">
-        <v>68</v>
+        <v>73</v>
       </c>
       <c r="D3" t="s">
-        <v>69</v>
+        <v>74</v>
       </c>
       <c r="F3" t="s">
-        <v>70</v>
+        <v>75</v>
       </c>
     </row>
     <row r="4" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
-        <v>71</v>
+        <v>76</v>
       </c>
       <c r="B4" t="s">
-        <v>63</v>
+        <v>68</v>
       </c>
       <c r="C4" t="s">
-        <v>72</v>
+        <v>77</v>
       </c>
       <c r="D4" t="s">
-        <v>73</v>
+        <v>78</v>
       </c>
       <c r="F4" t="s">
-        <v>74</v>
+        <v>79</v>
       </c>
     </row>
     <row r="5" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
-        <v>75</v>
+        <v>80</v>
       </c>
       <c r="B5" t="s">
-        <v>63</v>
+        <v>68</v>
       </c>
       <c r="C5" t="s">
-        <v>76</v>
+        <v>81</v>
       </c>
       <c r="D5" t="s">
-        <v>77</v>
+        <v>82</v>
       </c>
       <c r="F5" t="s">
-        <v>78</v>
+        <v>83</v>
+      </c>
+    </row>
+    <row r="6" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A6" t="s">
+        <v>84</v>
+      </c>
+      <c r="B6" t="s">
+        <v>68</v>
+      </c>
+      <c r="C6" t="s">
+        <v>85</v>
+      </c>
+      <c r="D6" t="s">
+        <v>86</v>
+      </c>
+      <c r="F6" t="s">
+        <v>87</v>
       </c>
     </row>
   </sheetData>
@@ -1968,33 +2052,33 @@
         <v>6</v>
       </c>
       <c r="D1" t="s">
-        <v>79</v>
+        <v>88</v>
       </c>
       <c r="E1" t="s">
         <v>8</v>
       </c>
       <c r="F1" t="s">
-        <v>80</v>
+        <v>89</v>
       </c>
       <c r="G1" t="s">
-        <v>81</v>
+        <v>90</v>
       </c>
     </row>
     <row r="2" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
-        <v>82</v>
+        <v>91</v>
       </c>
       <c r="B2" t="s">
-        <v>83</v>
+        <v>92</v>
       </c>
       <c r="C2" t="s">
-        <v>84</v>
+        <v>93</v>
       </c>
       <c r="D2" t="s">
-        <v>85</v>
+        <v>94</v>
       </c>
       <c r="E2" t="s">
-        <v>86</v>
+        <v>95</v>
       </c>
       <c r="F2">
         <v>1</v>
@@ -2005,19 +2089,19 @@
     </row>
     <row r="3" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
-        <v>87</v>
+        <v>96</v>
       </c>
       <c r="B3" t="s">
-        <v>83</v>
+        <v>92</v>
       </c>
       <c r="C3" t="s">
-        <v>88</v>
+        <v>97</v>
       </c>
       <c r="D3" t="s">
-        <v>89</v>
+        <v>98</v>
       </c>
       <c r="E3" t="s">
-        <v>90</v>
+        <v>99</v>
       </c>
       <c r="F3">
         <v>1</v>
@@ -2028,19 +2112,19 @@
     </row>
     <row r="4" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
-        <v>91</v>
+        <v>100</v>
       </c>
       <c r="B4" t="s">
-        <v>83</v>
+        <v>92</v>
       </c>
       <c r="C4" t="s">
-        <v>92</v>
+        <v>101</v>
       </c>
       <c r="D4" t="s">
-        <v>93</v>
+        <v>102</v>
       </c>
       <c r="E4" t="s">
-        <v>94</v>
+        <v>103</v>
       </c>
       <c r="F4">
         <v>1</v>
@@ -2048,19 +2132,19 @@
     </row>
     <row r="5" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
-        <v>95</v>
+        <v>104</v>
       </c>
       <c r="B5" t="s">
-        <v>83</v>
+        <v>92</v>
       </c>
       <c r="C5" t="s">
-        <v>96</v>
+        <v>105</v>
       </c>
       <c r="D5" t="s">
-        <v>97</v>
+        <v>106</v>
       </c>
       <c r="E5" t="s">
-        <v>98</v>
+        <v>107</v>
       </c>
       <c r="F5">
         <v>1</v>
@@ -2068,19 +2152,19 @@
     </row>
     <row r="6" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
-        <v>99</v>
+        <v>108</v>
       </c>
       <c r="B6" t="s">
-        <v>83</v>
+        <v>92</v>
       </c>
       <c r="C6" t="s">
-        <v>100</v>
+        <v>37</v>
       </c>
       <c r="D6" t="s">
-        <v>101</v>
+        <v>109</v>
       </c>
       <c r="E6" t="s">
-        <v>102</v>
+        <v>110</v>
       </c>
       <c r="F6">
         <v>1</v>
@@ -2088,19 +2172,19 @@
     </row>
     <row r="7" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
-        <v>103</v>
+        <v>111</v>
       </c>
       <c r="B7" t="s">
-        <v>83</v>
+        <v>92</v>
       </c>
       <c r="C7" t="s">
-        <v>104</v>
+        <v>112</v>
       </c>
       <c r="D7" t="s">
-        <v>105</v>
+        <v>113</v>
       </c>
       <c r="E7" t="s">
-        <v>106</v>
+        <v>114</v>
       </c>
       <c r="F7">
         <v>0</v>
@@ -2134,33 +2218,33 @@
         <v>6</v>
       </c>
       <c r="D1" t="s">
-        <v>107</v>
+        <v>115</v>
       </c>
       <c r="E1" t="s">
-        <v>108</v>
+        <v>116</v>
       </c>
       <c r="F1" t="s">
-        <v>109</v>
+        <v>117</v>
       </c>
       <c r="G1" t="s">
-        <v>110</v>
+        <v>118</v>
       </c>
       <c r="H1" t="s">
-        <v>80</v>
+        <v>89</v>
       </c>
       <c r="I1" t="s">
-        <v>81</v>
+        <v>90</v>
       </c>
       <c r="J1" t="s">
-        <v>79</v>
+        <v>88</v>
       </c>
     </row>
     <row r="2" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
-        <v>111</v>
+        <v>119</v>
       </c>
       <c r="B2" t="s">
-        <v>112</v>
+        <v>120</v>
       </c>
       <c r="C2" t="s">
         <v>2</v>
@@ -2169,13 +2253,13 @@
         <v>2</v>
       </c>
       <c r="E2" t="s">
-        <v>113</v>
+        <v>121</v>
       </c>
       <c r="F2" t="s">
-        <v>114</v>
+        <v>122</v>
       </c>
       <c r="G2" t="s">
-        <v>115</v>
+        <v>123</v>
       </c>
       <c r="H2">
         <v>1</v>
@@ -2186,10 +2270,10 @@
     </row>
     <row r="3" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
-        <v>116</v>
+        <v>124</v>
       </c>
       <c r="B3" t="s">
-        <v>112</v>
+        <v>120</v>
       </c>
       <c r="C3" t="s">
         <v>34</v>
@@ -2198,13 +2282,13 @@
         <v>34</v>
       </c>
       <c r="E3" t="s">
-        <v>117</v>
+        <v>125</v>
       </c>
       <c r="F3" t="s">
-        <v>114</v>
+        <v>122</v>
       </c>
       <c r="G3" t="s">
-        <v>118</v>
+        <v>126</v>
       </c>
       <c r="H3">
         <v>1</v>
@@ -2213,15 +2297,15 @@
         <v>1</v>
       </c>
       <c r="J3" t="s">
-        <v>119</v>
+        <v>127</v>
       </c>
     </row>
     <row r="4" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
+        <v>128</v>
+      </c>
+      <c r="B4" t="s">
         <v>120</v>
-      </c>
-      <c r="B4" t="s">
-        <v>112</v>
       </c>
       <c r="C4" t="s">
         <v>18</v>
@@ -2230,13 +2314,13 @@
         <v>18</v>
       </c>
       <c r="E4" t="s">
-        <v>121</v>
+        <v>129</v>
       </c>
       <c r="F4" t="s">
-        <v>114</v>
+        <v>122</v>
       </c>
       <c r="G4" t="s">
-        <v>122</v>
+        <v>130</v>
       </c>
       <c r="H4">
         <v>1</v>
@@ -2247,10 +2331,10 @@
     </row>
     <row r="5" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
-        <v>123</v>
+        <v>131</v>
       </c>
       <c r="B5" t="s">
-        <v>112</v>
+        <v>120</v>
       </c>
       <c r="C5" t="s">
         <v>6</v>
@@ -2259,13 +2343,13 @@
         <v>6</v>
       </c>
       <c r="E5" t="s">
-        <v>124</v>
+        <v>132</v>
       </c>
       <c r="F5" t="s">
-        <v>118</v>
+        <v>126</v>
       </c>
       <c r="G5" t="s">
-        <v>125</v>
+        <v>133</v>
       </c>
       <c r="H5">
         <v>1</v>
@@ -2274,15 +2358,15 @@
         <v>1</v>
       </c>
       <c r="J5" t="s">
-        <v>126</v>
+        <v>134</v>
       </c>
     </row>
     <row r="6" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
-        <v>127</v>
+        <v>135</v>
       </c>
       <c r="B6" t="s">
-        <v>112</v>
+        <v>120</v>
       </c>
       <c r="C6" t="s">
         <v>8</v>
@@ -2291,56 +2375,56 @@
         <v>8</v>
       </c>
       <c r="E6" t="s">
-        <v>128</v>
+        <v>136</v>
       </c>
       <c r="F6" t="s">
-        <v>118</v>
+        <v>126</v>
       </c>
       <c r="G6" t="s">
-        <v>125</v>
+        <v>133</v>
       </c>
       <c r="H6">
         <v>1</v>
       </c>
       <c r="J6" t="s">
-        <v>129</v>
+        <v>137</v>
       </c>
     </row>
     <row r="7" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
-        <v>130</v>
+        <v>138</v>
       </c>
       <c r="B7" t="s">
-        <v>112</v>
+        <v>120</v>
       </c>
       <c r="C7" t="s">
-        <v>131</v>
+        <v>139</v>
       </c>
       <c r="D7" t="s">
-        <v>131</v>
+        <v>139</v>
       </c>
       <c r="E7" t="s">
-        <v>132</v>
+        <v>140</v>
       </c>
       <c r="F7" t="s">
-        <v>118</v>
+        <v>126</v>
       </c>
       <c r="G7" t="s">
-        <v>133</v>
+        <v>141</v>
       </c>
       <c r="H7">
         <v>1</v>
       </c>
       <c r="J7" t="s">
-        <v>134</v>
+        <v>142</v>
       </c>
     </row>
     <row r="8" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A8" t="s">
-        <v>135</v>
+        <v>143</v>
       </c>
       <c r="B8" t="s">
-        <v>112</v>
+        <v>120</v>
       </c>
       <c r="C8" t="s">
         <v>18</v>
@@ -2349,13 +2433,13 @@
         <v>18</v>
       </c>
       <c r="E8" t="s">
-        <v>136</v>
+        <v>144</v>
       </c>
       <c r="F8" t="s">
-        <v>118</v>
+        <v>126</v>
       </c>
       <c r="G8" t="s">
-        <v>137</v>
+        <v>145</v>
       </c>
       <c r="H8">
         <v>1</v>
@@ -2363,10 +2447,10 @@
     </row>
     <row r="9" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A9" t="s">
-        <v>138</v>
+        <v>146</v>
       </c>
       <c r="B9" t="s">
-        <v>112</v>
+        <v>120</v>
       </c>
       <c r="C9" t="s">
         <v>6</v>
@@ -2375,14 +2459,14 @@
         <v>6</v>
       </c>
       <c r="E9" t="s">
-        <v>139</v>
+        <v>147</v>
       </c>
       <c r="F9" t="s">
+        <v>141</v>
+      </c>
+      <c r="G9" t="s">
         <v>133</v>
       </c>
-      <c r="G9" t="s">
-        <v>125</v>
-      </c>
       <c r="H9">
         <v>1</v>
       </c>
@@ -2390,15 +2474,15 @@
         <v>1</v>
       </c>
       <c r="J9" t="s">
-        <v>126</v>
+        <v>134</v>
       </c>
     </row>
     <row r="10" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A10" t="s">
-        <v>140</v>
+        <v>148</v>
       </c>
       <c r="B10" t="s">
-        <v>112</v>
+        <v>120</v>
       </c>
       <c r="C10" t="s">
         <v>8</v>
@@ -2407,42 +2491,42 @@
         <v>8</v>
       </c>
       <c r="E10" t="s">
+        <v>149</v>
+      </c>
+      <c r="F10" t="s">
         <v>141</v>
       </c>
-      <c r="F10" t="s">
+      <c r="G10" t="s">
         <v>133</v>
       </c>
-      <c r="G10" t="s">
-        <v>125</v>
-      </c>
       <c r="H10">
         <v>1</v>
       </c>
       <c r="J10" t="s">
-        <v>129</v>
+        <v>137</v>
       </c>
     </row>
     <row r="11" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A11" t="s">
-        <v>142</v>
+        <v>150</v>
       </c>
       <c r="B11" t="s">
-        <v>112</v>
+        <v>120</v>
       </c>
       <c r="C11" t="s">
-        <v>143</v>
+        <v>151</v>
       </c>
       <c r="D11" t="s">
-        <v>143</v>
+        <v>151</v>
       </c>
       <c r="E11" t="s">
-        <v>144</v>
+        <v>152</v>
       </c>
       <c r="F11" t="s">
-        <v>133</v>
+        <v>141</v>
       </c>
       <c r="G11" t="s">
-        <v>118</v>
+        <v>126</v>
       </c>
       <c r="H11">
         <v>1</v>
@@ -2451,30 +2535,30 @@
         <v>1</v>
       </c>
       <c r="J11" t="s">
-        <v>145</v>
+        <v>153</v>
       </c>
     </row>
     <row r="12" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A12" t="s">
-        <v>146</v>
+        <v>154</v>
       </c>
       <c r="B12" t="s">
-        <v>112</v>
+        <v>120</v>
       </c>
       <c r="C12" t="s">
-        <v>147</v>
+        <v>155</v>
       </c>
       <c r="D12" t="s">
-        <v>147</v>
+        <v>155</v>
       </c>
       <c r="E12" t="s">
-        <v>148</v>
+        <v>156</v>
       </c>
       <c r="F12" t="s">
-        <v>133</v>
+        <v>141</v>
       </c>
       <c r="G12" t="s">
-        <v>149</v>
+        <v>157</v>
       </c>
       <c r="H12">
         <v>1</v>
@@ -2483,31 +2567,31 @@
         <v>1</v>
       </c>
       <c r="J12" t="s">
-        <v>150</v>
+        <v>158</v>
       </c>
     </row>
     <row r="13" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A13" t="s">
-        <v>151</v>
+        <v>159</v>
       </c>
       <c r="B13" t="s">
-        <v>112</v>
+        <v>120</v>
       </c>
       <c r="C13" t="s">
-        <v>152</v>
+        <v>160</v>
       </c>
       <c r="D13" t="s">
-        <v>152</v>
+        <v>160</v>
       </c>
       <c r="E13" t="s">
-        <v>153</v>
+        <v>161</v>
       </c>
       <c r="F13" t="s">
+        <v>141</v>
+      </c>
+      <c r="G13" t="s">
         <v>133</v>
       </c>
-      <c r="G13" t="s">
-        <v>125</v>
-      </c>
       <c r="H13">
         <v>1</v>
       </c>
@@ -2515,15 +2599,15 @@
         <v>1</v>
       </c>
       <c r="J13" t="s">
-        <v>154</v>
+        <v>162</v>
       </c>
     </row>
     <row r="14" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A14" t="s">
-        <v>155</v>
+        <v>163</v>
       </c>
       <c r="B14" t="s">
-        <v>112</v>
+        <v>120</v>
       </c>
       <c r="C14" t="s">
         <v>16</v>
@@ -2532,13 +2616,13 @@
         <v>16</v>
       </c>
       <c r="E14" t="s">
-        <v>156</v>
+        <v>164</v>
       </c>
       <c r="F14" t="s">
-        <v>133</v>
+        <v>141</v>
       </c>
       <c r="G14" t="s">
-        <v>157</v>
+        <v>165</v>
       </c>
       <c r="H14">
         <v>1</v>
@@ -2547,30 +2631,30 @@
         <v>1</v>
       </c>
       <c r="J14" t="s">
-        <v>158</v>
+        <v>166</v>
       </c>
     </row>
     <row r="15" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A15" t="s">
-        <v>159</v>
+        <v>167</v>
       </c>
       <c r="B15" t="s">
-        <v>112</v>
+        <v>120</v>
       </c>
       <c r="C15" t="s">
-        <v>160</v>
+        <v>168</v>
       </c>
       <c r="D15" t="s">
-        <v>160</v>
+        <v>168</v>
       </c>
       <c r="E15" t="s">
-        <v>161</v>
+        <v>169</v>
       </c>
       <c r="F15" t="s">
-        <v>133</v>
+        <v>141</v>
       </c>
       <c r="G15" t="s">
-        <v>162</v>
+        <v>170</v>
       </c>
       <c r="H15">
         <v>0</v>
@@ -2579,30 +2663,30 @@
         <v>1</v>
       </c>
       <c r="J15" t="s">
-        <v>163</v>
+        <v>171</v>
       </c>
     </row>
     <row r="16" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A16" t="s">
-        <v>164</v>
+        <v>172</v>
       </c>
       <c r="B16" t="s">
-        <v>112</v>
+        <v>120</v>
       </c>
       <c r="C16" t="s">
-        <v>165</v>
+        <v>173</v>
       </c>
       <c r="D16" t="s">
-        <v>165</v>
+        <v>173</v>
       </c>
       <c r="E16" t="s">
-        <v>166</v>
+        <v>174</v>
       </c>
       <c r="F16" t="s">
+        <v>141</v>
+      </c>
+      <c r="G16" t="s">
         <v>133</v>
-      </c>
-      <c r="G16" t="s">
-        <v>125</v>
       </c>
       <c r="H16">
         <v>1</v>
@@ -2613,25 +2697,25 @@
     </row>
     <row r="17" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A17" t="s">
-        <v>167</v>
+        <v>175</v>
       </c>
       <c r="B17" t="s">
-        <v>112</v>
+        <v>120</v>
       </c>
       <c r="C17" t="s">
-        <v>168</v>
+        <v>176</v>
       </c>
       <c r="D17" t="s">
-        <v>168</v>
+        <v>176</v>
       </c>
       <c r="E17" t="s">
-        <v>169</v>
+        <v>177</v>
       </c>
       <c r="F17" t="s">
+        <v>141</v>
+      </c>
+      <c r="G17" t="s">
         <v>133</v>
-      </c>
-      <c r="G17" t="s">
-        <v>125</v>
       </c>
       <c r="H17">
         <v>0</v>
@@ -2642,25 +2726,25 @@
     </row>
     <row r="18" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A18" t="s">
-        <v>170</v>
+        <v>178</v>
       </c>
       <c r="B18" t="s">
-        <v>112</v>
+        <v>120</v>
       </c>
       <c r="C18" t="s">
-        <v>171</v>
+        <v>179</v>
       </c>
       <c r="D18" t="s">
-        <v>171</v>
+        <v>179</v>
       </c>
       <c r="E18" t="s">
-        <v>172</v>
+        <v>180</v>
       </c>
       <c r="F18" t="s">
+        <v>141</v>
+      </c>
+      <c r="G18" t="s">
         <v>133</v>
-      </c>
-      <c r="G18" t="s">
-        <v>125</v>
       </c>
       <c r="H18">
         <v>0</v>
@@ -2671,25 +2755,25 @@
     </row>
     <row r="19" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A19" t="s">
-        <v>173</v>
+        <v>181</v>
       </c>
       <c r="B19" t="s">
-        <v>112</v>
+        <v>120</v>
       </c>
       <c r="C19" t="s">
-        <v>174</v>
+        <v>182</v>
       </c>
       <c r="D19" t="s">
-        <v>174</v>
+        <v>182</v>
       </c>
       <c r="E19" t="s">
-        <v>175</v>
+        <v>183</v>
       </c>
       <c r="F19" t="s">
+        <v>141</v>
+      </c>
+      <c r="G19" t="s">
         <v>133</v>
-      </c>
-      <c r="G19" t="s">
-        <v>125</v>
       </c>
       <c r="H19">
         <v>0</v>
@@ -2700,25 +2784,25 @@
     </row>
     <row r="20" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A20" t="s">
-        <v>176</v>
+        <v>184</v>
       </c>
       <c r="B20" t="s">
-        <v>112</v>
+        <v>120</v>
       </c>
       <c r="C20" t="s">
-        <v>177</v>
+        <v>185</v>
       </c>
       <c r="D20" t="s">
-        <v>177</v>
+        <v>185</v>
       </c>
       <c r="E20" t="s">
-        <v>178</v>
+        <v>186</v>
       </c>
       <c r="F20" t="s">
+        <v>141</v>
+      </c>
+      <c r="G20" t="s">
         <v>133</v>
-      </c>
-      <c r="G20" t="s">
-        <v>125</v>
       </c>
       <c r="H20">
         <v>0</v>
@@ -2729,25 +2813,25 @@
     </row>
     <row r="21" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A21" t="s">
-        <v>179</v>
+        <v>187</v>
       </c>
       <c r="B21" t="s">
-        <v>112</v>
+        <v>120</v>
       </c>
       <c r="C21" t="s">
-        <v>180</v>
+        <v>188</v>
       </c>
       <c r="D21" t="s">
-        <v>180</v>
+        <v>188</v>
       </c>
       <c r="E21" t="s">
-        <v>181</v>
+        <v>189</v>
       </c>
       <c r="F21" t="s">
-        <v>133</v>
+        <v>141</v>
       </c>
       <c r="G21" t="s">
-        <v>162</v>
+        <v>170</v>
       </c>
       <c r="H21">
         <v>0</v>
@@ -2758,25 +2842,25 @@
     </row>
     <row r="22" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A22" t="s">
-        <v>182</v>
+        <v>190</v>
       </c>
       <c r="B22" t="s">
-        <v>112</v>
+        <v>120</v>
       </c>
       <c r="C22" t="s">
-        <v>183</v>
+        <v>191</v>
       </c>
       <c r="D22" t="s">
-        <v>183</v>
+        <v>191</v>
       </c>
       <c r="E22" t="s">
-        <v>184</v>
+        <v>192</v>
       </c>
       <c r="F22" t="s">
-        <v>133</v>
+        <v>141</v>
       </c>
       <c r="G22" t="s">
-        <v>162</v>
+        <v>170</v>
       </c>
       <c r="H22">
         <v>0</v>
@@ -2787,25 +2871,25 @@
     </row>
     <row r="23" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A23" t="s">
-        <v>185</v>
+        <v>193</v>
       </c>
       <c r="B23" t="s">
-        <v>112</v>
+        <v>120</v>
       </c>
       <c r="C23" t="s">
-        <v>186</v>
+        <v>194</v>
       </c>
       <c r="D23" t="s">
-        <v>186</v>
+        <v>194</v>
       </c>
       <c r="E23" t="s">
-        <v>187</v>
+        <v>195</v>
       </c>
       <c r="F23" t="s">
-        <v>133</v>
+        <v>141</v>
       </c>
       <c r="G23" t="s">
-        <v>162</v>
+        <v>170</v>
       </c>
       <c r="H23">
         <v>0</v>
@@ -2816,10 +2900,10 @@
     </row>
     <row r="24" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A24" t="s">
-        <v>188</v>
+        <v>196</v>
       </c>
       <c r="B24" t="s">
-        <v>112</v>
+        <v>120</v>
       </c>
       <c r="C24" t="s">
         <v>6</v>
@@ -2828,13 +2912,13 @@
         <v>6</v>
       </c>
       <c r="E24" t="s">
-        <v>189</v>
+        <v>197</v>
       </c>
       <c r="F24" t="s">
-        <v>149</v>
+        <v>157</v>
       </c>
       <c r="G24" t="s">
-        <v>125</v>
+        <v>133</v>
       </c>
       <c r="H24">
         <v>1</v>
@@ -2843,15 +2927,15 @@
         <v>1</v>
       </c>
       <c r="J24" t="s">
-        <v>126</v>
+        <v>134</v>
       </c>
     </row>
     <row r="25" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A25" t="s">
-        <v>190</v>
+        <v>198</v>
       </c>
       <c r="B25" t="s">
-        <v>112</v>
+        <v>120</v>
       </c>
       <c r="C25" t="s">
         <v>8</v>
@@ -2860,42 +2944,42 @@
         <v>8</v>
       </c>
       <c r="E25" t="s">
-        <v>191</v>
+        <v>199</v>
       </c>
       <c r="F25" t="s">
-        <v>149</v>
+        <v>157</v>
       </c>
       <c r="G25" t="s">
-        <v>125</v>
+        <v>133</v>
       </c>
       <c r="H25">
         <v>0</v>
       </c>
       <c r="J25" t="s">
-        <v>129</v>
+        <v>137</v>
       </c>
     </row>
     <row r="26" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A26" t="s">
-        <v>192</v>
+        <v>200</v>
       </c>
       <c r="B26" t="s">
-        <v>112</v>
+        <v>120</v>
       </c>
       <c r="C26" t="s">
-        <v>193</v>
+        <v>201</v>
       </c>
       <c r="D26" t="s">
-        <v>193</v>
+        <v>201</v>
       </c>
       <c r="E26" t="s">
-        <v>194</v>
+        <v>202</v>
       </c>
       <c r="F26" t="s">
-        <v>162</v>
+        <v>170</v>
       </c>
       <c r="G26" t="s">
-        <v>133</v>
+        <v>141</v>
       </c>
       <c r="H26">
         <v>0</v>
@@ -2904,15 +2988,15 @@
         <v>1</v>
       </c>
       <c r="J26" t="s">
-        <v>195</v>
+        <v>203</v>
       </c>
     </row>
     <row r="27" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A27" t="s">
-        <v>196</v>
+        <v>204</v>
       </c>
       <c r="B27" t="s">
-        <v>112</v>
+        <v>120</v>
       </c>
       <c r="C27" t="s">
         <v>33</v>
@@ -2921,13 +3005,13 @@
         <v>33</v>
       </c>
       <c r="E27" t="s">
-        <v>197</v>
+        <v>205</v>
       </c>
       <c r="F27" t="s">
-        <v>198</v>
+        <v>206</v>
       </c>
       <c r="G27" t="s">
-        <v>199</v>
+        <v>207</v>
       </c>
       <c r="H27">
         <v>1</v>
@@ -2936,15 +3020,15 @@
         <v>1</v>
       </c>
       <c r="J27" t="s">
-        <v>200</v>
+        <v>208</v>
       </c>
     </row>
     <row r="28" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A28" t="s">
-        <v>201</v>
+        <v>209</v>
       </c>
       <c r="B28" t="s">
-        <v>112</v>
+        <v>120</v>
       </c>
       <c r="C28" t="s">
         <v>34</v>
@@ -2953,13 +3037,13 @@
         <v>34</v>
       </c>
       <c r="E28" t="s">
-        <v>202</v>
+        <v>210</v>
       </c>
       <c r="F28" t="s">
-        <v>198</v>
+        <v>206</v>
       </c>
       <c r="G28" t="s">
-        <v>118</v>
+        <v>126</v>
       </c>
       <c r="H28">
         <v>1</v>
@@ -2968,7 +3052,7 @@
         <v>1</v>
       </c>
       <c r="J28" t="s">
-        <v>119</v>
+        <v>127</v>
       </c>
     </row>
   </sheetData>

</xml_diff>